<commit_message>
Actualizacion plantilla login y Pacientes
</commit_message>
<xml_diff>
--- a/01-Test-Cases/Login_Test_Cases.xlsx
+++ b/01-Test-Cases/Login_Test_Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Desktop\Trabajos Personal\QA-testing-gestion-turnos-medicos\01-Test-Cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE2B944A-16DC-4F50-9E41-299CBCF85DB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC389BCB-D6E7-4383-95B7-C7B11704E062}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{91C9C9F2-8AA2-4FDE-9D3F-0B1C8967849F}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="92">
   <si>
     <t>ID</t>
   </si>
@@ -117,9 +117,6 @@
     <t>El usuario debe estar regristrado y activo en el sistema.</t>
   </si>
   <si>
-    <t>Iniciar sesión con credencial válidas.</t>
-  </si>
-  <si>
     <t>Ninguna</t>
   </si>
   <si>
@@ -142,13 +139,233 @@
   </si>
   <si>
     <t>El sistema rechaza la autenticación y muestra un mensaje indicando que las credenciales son incorrectas.</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-003</t>
+  </si>
+  <si>
+    <t>Intentar iniciar sesión con un usuario inexistente</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-004</t>
+  </si>
+  <si>
+    <t>Ingresar un usuario con espacios al inicio o al final</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-005</t>
+  </si>
+  <si>
+    <t>Ingresar una contraseña con espacios al inicio o al final</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-006</t>
+  </si>
+  <si>
+    <t>Intentar iniciar sesión con ambos campos vacíos</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-007</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Intentar iniciar sesión con el campo </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Usuario</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> vacío</t>
+    </r>
+  </si>
+  <si>
+    <t>TC-LOGIN-008</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Intentar iniciar sesión con el campo </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Contraseña</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> vacío</t>
+    </r>
+  </si>
+  <si>
+    <t>Cerrar sesión correctamente</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-009</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-010</t>
+  </si>
+  <si>
+    <t>Intentar acceder al sistema sin haber iniciado sesión</t>
+  </si>
+  <si>
+    <t>Media</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-011</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-012</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-013</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-014</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-015</t>
+  </si>
+  <si>
+    <t>Ingresar un usuario que supere la longitud máxima permitida</t>
+  </si>
+  <si>
+    <t>Ingresar una contraseña que supere la longitud máxima permitida</t>
+  </si>
+  <si>
+    <t>Verificar que la contraseña se muestre oculta (con puntos o asteriscos)</t>
+  </si>
+  <si>
+    <t>Verificar que el botón Ingresar funcione al presionar la tecla Enter</t>
+  </si>
+  <si>
+    <t>Verificar que se muestre un mensaje de error claro cuando las credenciales son incorrectas</t>
+  </si>
+  <si>
+    <t>El usuario no debe estar regristado en el sistema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Abrir el sistema.                                  2. Ingresar un usuario con espacio delante y/o final.                                          3. Ingresar contraseña correcta                                   4. Presionar ingresar.    </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Abrir el sistema.                                  2. Ingresar un usuario válido.                                          3. Ingresar contraseña correcta  con espacio delante y/o final.                                  4. Presionar ingresar.    </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Abrir el sistema.                                                                   2. Presionar ingresar.    </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Abrir el sistema.                                  2. Ingresar contraseña válida.                             3. Presionar ingresar.    </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Abrir el sistema.                                  2. Ingresar datos tanto usuario como contraseña no regristrados.                                          3. Presionar el boton ingresar.    </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Abrir el sistema.                                  2. Ingresar nombre de usuario.                             3. Presionar ingresar.    </t>
+  </si>
+  <si>
+    <t>El sistema muestra un mensaje indicando que los campos estan vacíos.</t>
+  </si>
+  <si>
+    <t>El sistema muestra un mensaje indicando que el campo "Constraseña" esta vacío y rechaza la autenticación.</t>
+  </si>
+  <si>
+    <t>El sistema muestra un mensaje indicando que el campo "Usuario" esta vacío y rechaza la autenticación.</t>
+  </si>
+  <si>
+    <t>No aplica.</t>
+  </si>
+  <si>
+    <t>Iniciar sesión con credenciales válidas.</t>
+  </si>
+  <si>
+    <t>El sistema procesa el usuario según la regla definida para espacios en blanco y permite o rechaza el acceso de acuerdo con esa especificación</t>
+  </si>
+  <si>
+    <t>El sistema rechaza la autenticación y muestra un mensaje indicando que el usuario o la contraseña son incorrectos.</t>
+  </si>
+  <si>
+    <t>El usuario debe haber iniciado sesión correctamente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Iniciar sesión con un usuario válido.                                           2.Presionar el botón Salir o Cerrar sesión.          </t>
+  </si>
+  <si>
+    <t>El sistema cierra la sesión del usuario y redirige a la pantalla de inicio de sesión.</t>
+  </si>
+  <si>
+    <t>El usuario no debe haber iniciado sesión.</t>
+  </si>
+  <si>
+    <t>1. Intentar acceder directamente a una página protegida del sistema (por ejemplo, /dashboard o una URL interna).</t>
+  </si>
+  <si>
+    <t>El sistema impide el acceso y redirige al usuario a la pantalla de inicio de sesión o muestra un mensaje indicando que debe autenticarse.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Abrir el sistema.                                  2. Ingresar un nombre de usuario con una longitud superior a la permitida.                                         3. Ingresar una contraseña válida.                                           4. Presionar ingresar.    </t>
+  </si>
+  <si>
+    <t>El sistema valida la longitud del campo usuario y muestra un mensaje de error o impide ingresar más caracteres, según la especificación.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Abrir el sistema.                                  2. Ingresar un usuario válido.                         3. Ingresar una contraseña con una longitud superior a la permitida.                                          4. Presionar ingresar.    </t>
+  </si>
+  <si>
+    <t>El sistema valida la longitud del campo contraseña y muestra un mensaje de error o impide ingresar más caracteres, según la especificación.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Abrir el sistema.                                  2. Posicionarse sobre el campo Contraseña.                                  3. Escribir una contraseña.   </t>
+  </si>
+  <si>
+    <t>Los caracteres ingresados en el campo contraseña se muestran ocultos (por ejemplo, mediante puntos o asteriscos) para proteger la información del usuario.</t>
+  </si>
+  <si>
+    <t>El usuario debe estar registrado y activo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Abrir el sistema.                                  2. Ingresar un usuario válido.                                          3. Ingresar una contraseña válida.                                           4. Presionar la tecla ENTER sin hacer click en el boton  ingresar. </t>
+  </si>
+  <si>
+    <t>El sistema inicia sesión correctamente y muestra la pantalla principal del usuario.</t>
+  </si>
+  <si>
+    <t>1. Abrir el sistema.                                  2. Ingresar un usuario válido.                                          3. Ingresar una contraseña incorrecta.                                           4. Presionar ingresar.</t>
+  </si>
+  <si>
+    <t>El sistema muestra un mensaje de error claro e informativo indicando que las credenciales ingresadas son incorrectas, sin revelar información sensible sobre la existencia del usuario.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -168,6 +385,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -199,7 +422,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -218,6 +441,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -538,8 +764,8 @@
   <cols>
     <col min="2" max="2" width="17" customWidth="1"/>
     <col min="3" max="3" width="38.85546875" customWidth="1"/>
-    <col min="4" max="4" width="23.5703125" customWidth="1"/>
-    <col min="5" max="5" width="49.140625" customWidth="1"/>
+    <col min="4" max="4" width="34.5703125" customWidth="1"/>
+    <col min="5" max="5" width="27" customWidth="1"/>
     <col min="6" max="6" width="29.5703125" customWidth="1"/>
     <col min="7" max="7" width="32.5703125" customWidth="1"/>
     <col min="8" max="8" width="27.28515625" customWidth="1"/>
@@ -547,10 +773,8 @@
     <col min="11" max="11" width="16.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>13</v>
       </c>
@@ -558,7 +782,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
         <v>15</v>
       </c>
@@ -566,7 +790,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
@@ -574,7 +798,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
         <v>18</v>
       </c>
@@ -582,7 +806,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
         <v>20</v>
       </c>
@@ -590,7 +814,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
         <v>22</v>
       </c>
@@ -598,80 +822,83 @@
         <v>46234</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>2</v>
+      </c>
       <c r="B10" s="1" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K10" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>23</v>
+      </c>
       <c r="B11" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G11" s="6" t="s">
+      <c r="B12" s="6" t="s">
         <v>29</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="K11" s="6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="75" x14ac:dyDescent="0.25">
-      <c r="B12" s="6" t="s">
-        <v>23</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>30</v>
       </c>
       <c r="D12" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="6" t="s">
         <v>31</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>11</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>32</v>
@@ -679,327 +906,480 @@
       <c r="G12" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="H12" s="6" t="s">
+      <c r="H12" s="6"/>
+      <c r="I12" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6" t="s">
+      <c r="C13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="K12" s="6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6" t="s">
+      <c r="J13" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H15" s="6"/>
+      <c r="I15" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6" t="s">
+      <c r="E16" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="H16" s="6"/>
+      <c r="I16" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="K13" s="6"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6" t="s">
+      <c r="J16" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6" t="s">
+      <c r="E17" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="H17" s="6"/>
+      <c r="I17" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="K14" s="6"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6" t="s">
+      <c r="J17" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6" t="s">
+      <c r="E18" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="H18" s="6"/>
+      <c r="I18" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="K15" s="6"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6" t="s">
+      <c r="J18" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="6"/>
-      <c r="J16" s="6" t="s">
+      <c r="E19" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="K16" s="6"/>
-    </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6" t="s">
+      <c r="J19" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D20" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="6"/>
-      <c r="J17" s="6" t="s">
+      <c r="E20" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="H20" s="6"/>
+      <c r="I20" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="K17" s="6"/>
-    </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6" t="s">
+      <c r="J20" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="105" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="H21" s="6"/>
+      <c r="I21" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="H22" s="6"/>
+      <c r="I22" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="J22" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D23" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="6"/>
-      <c r="J18" s="6" t="s">
+      <c r="E23" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="K18" s="6"/>
-    </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6" t="s">
+      <c r="J23" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="105" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D24" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="6" t="s">
+      <c r="E24" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="K19" s="6"/>
-    </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6" t="s">
+      <c r="J24" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D25" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="6"/>
-      <c r="I20" s="6"/>
-      <c r="J20" s="6" t="s">
+      <c r="E25" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="K20" s="6"/>
-    </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
-      <c r="J21" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="K21" s="6"/>
-    </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
-      <c r="I22" s="6"/>
-      <c r="J22" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="K22" s="6"/>
-    </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="K23" s="6"/>
-    </row>
-    <row r="24" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
-      <c r="I24" s="6"/>
-      <c r="J24" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="K24" s="6"/>
-    </row>
-    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6"/>
-      <c r="I25" s="6"/>
       <c r="J25" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="K25" s="6"/>
-    </row>
-    <row r="26" spans="2:11" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
-      <c r="E26" s="6" t="s">
-        <v>11</v>
-      </c>
+      <c r="E26" s="6"/>
       <c r="F26" s="6"/>
       <c r="G26" s="6"/>
       <c r="H26" s="6"/>
       <c r="I26" s="6"/>
-      <c r="J26" s="6" t="s">
-        <v>12</v>
-      </c>
+      <c r="J26" s="6"/>
       <c r="K26" s="6"/>
     </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
-      <c r="E27" s="6" t="s">
-        <v>11</v>
-      </c>
+      <c r="E27" s="6"/>
       <c r="F27" s="6"/>
       <c r="G27" s="6"/>
       <c r="H27" s="6"/>
       <c r="I27" s="6"/>
-      <c r="J27" s="6" t="s">
-        <v>12</v>
-      </c>
+      <c r="J27" s="6"/>
       <c r="K27" s="6"/>
     </row>
-    <row r="28" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B28" s="6"/>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
-      <c r="E28" s="6" t="s">
-        <v>11</v>
-      </c>
+      <c r="E28" s="6"/>
       <c r="F28" s="6"/>
       <c r="G28" s="6"/>
       <c r="H28" s="6"/>
       <c r="I28" s="6"/>
-      <c r="J28" s="6" t="s">
-        <v>12</v>
-      </c>
+      <c r="J28" s="6"/>
       <c r="K28" s="6"/>
     </row>
-    <row r="29" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B29" s="6"/>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
-      <c r="E29" s="6" t="s">
-        <v>11</v>
-      </c>
+      <c r="E29" s="6"/>
       <c r="F29" s="6"/>
       <c r="G29" s="6"/>
       <c r="H29" s="6"/>
       <c r="I29" s="6"/>
-      <c r="J29" s="6" t="s">
-        <v>12</v>
-      </c>
+      <c r="J29" s="6"/>
       <c r="K29" s="6"/>
     </row>
-    <row r="30" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B30" s="6"/>
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
-      <c r="E30" s="6" t="s">
-        <v>11</v>
-      </c>
+      <c r="E30" s="6"/>
       <c r="F30" s="6"/>
       <c r="G30" s="6"/>
       <c r="H30" s="6"/>
       <c r="I30" s="6"/>
-      <c r="J30" s="6" t="s">
-        <v>12</v>
-      </c>
+      <c r="J30" s="6"/>
       <c r="K30" s="6"/>
     </row>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B31" s="6"/>
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
-      <c r="E31" s="6" t="s">
-        <v>11</v>
-      </c>
+      <c r="E31" s="6"/>
       <c r="F31" s="6"/>
       <c r="G31" s="6"/>
       <c r="H31" s="6"/>
       <c r="I31" s="6"/>
-      <c r="J31" s="6" t="s">
-        <v>12</v>
-      </c>
+      <c r="J31" s="6"/>
       <c r="K31" s="6"/>
     </row>
-    <row r="32" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B32" s="6"/>
       <c r="C32" s="6"/>
-      <c r="E32" s="6" t="s">
-        <v>11</v>
-      </c>
+      <c r="E32" s="6"/>
       <c r="F32" s="6"/>
       <c r="G32" s="6"/>
       <c r="H32" s="6"/>
@@ -1010,9 +1390,7 @@
     <row r="33" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B33" s="6"/>
       <c r="C33" s="6"/>
-      <c r="E33" s="6" t="s">
-        <v>11</v>
-      </c>
+      <c r="E33" s="6"/>
       <c r="F33" s="6"/>
       <c r="G33" s="6"/>
       <c r="H33" s="6"/>
@@ -1076,11 +1454,12 @@
       <c r="J38" s="5"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E11:E33" xr:uid="{2495E873-81AD-4B06-A3F9-0E076BF3AAC6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E26:E33 D11:D25" xr:uid="{2495E873-81AD-4B06-A3F9-0E076BF3AAC6}">
       <formula1>"Alta, Media, Baja"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J11:J31" xr:uid="{EF00B5E8-DCB1-42B7-99B2-94FBD39C66E4}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J26:J31 I11:I25" xr:uid="{EF00B5E8-DCB1-42B7-99B2-94FBD39C66E4}">
       <formula1>"Pendiente, En ejecución, Aprobado, Falló, Bloqueado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>